<commit_message>
fix(news): update 2026-10-21 verified coverage
Replace overlapping 10/21 content with a distinct daily set and regenerate related workbook/version outputs.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/exports/day-2026-10-21-en.xlsx
+++ b/docs/exports/day-2026-10-21-en.xlsx
@@ -552,7 +552,7 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Malaysia AI-facility commitments and delivery milestones remain distinct
+            <t xml:space="preserve">Malaysia approves 27 data-center projects worth about US$55.4 billion
 </t>
           </r>
           <r>
@@ -561,15 +561,15 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>Bitdeer’s A201 in Malaysia still distinguishes site readiness in January 2027 from full deployment in April 2027, while Aolani’s disclosure is only a non-binding LOI covering up to 500 MW. Both cases show that AI-facility progress is measured separately by contracted coverage, site completion and power readiness, and cannot be treated as installed capacity.</t>
+            <t>Regional coverage reviewed on October 21 says Malaysia has approved 27 additional data-center projects worth about US$55.4 billion. The figure reflects approvals and investment commitments rather than same-day energization, rack deployment, and commercial operations; supply-chain impact still depends on construction, substation, and tenant ramp timing.</t>
           </r>
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>46315</v>
-      </c>
-    </row>
-    <row r="4" ht="98" customHeight="1">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="4" ht="82" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>02</t>
@@ -584,7 +584,7 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">MiTAC’s new-factory and expansion plan is public, but capacity timing is not yet defined
+            <t xml:space="preserve">Peninsular Malaysia data-center demand estimated at 8,391MW by 2030, with Johor above half
 </t>
           </r>
           <r>
@@ -593,12 +593,12 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>MiTAC disclosed approximately NT$12.62 billion in Taiwan investment covering a new Yangmei plant and expansions in Zhunan and Linkou, but did not publish the equipment-install timing or acceptance thresholds for each site. The project remains a planned capital expansion rather than an immediate shipped or live capacity figure.</t>
+            <t>October 21 reporting indicates Peninsular Malaysia data-center demand could reach 8,391MW by 2030, with Johor accounting for more than half. This is a demand estimate rather than current load; real supply-chain effects still depend on grid upgrades, interconnection approvals, and phased commissioning.</t>
           </r>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="5" ht="118" customHeight="1">
@@ -616,7 +616,7 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">TPK and PTI packaging equipment and glass-substrate validation still center on pilot runs and customer acceptance
+            <t xml:space="preserve">Vietnam electronics expansion signals strengthen, with multi-billion-dollar intentions still pending execution
 </t>
           </r>
           <r>
@@ -625,12 +625,12 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>TPK outlines a two-year NT$6 billion TGV plan, while PTI discloses nearby equipment procurement and packaging-validation milestones. Both actions emphasize validation, scale-up and customer-fit, but they do not yet amount to production readiness, because equipment purchase, pilot production and customer acceptance are separate milestones.</t>
+            <t>Supply-chain coverage reviewed on October 21 highlights continued multi-billion-dollar investment intentions in Vietnam’s electronics and chip-testing chain, including Taiwanese and Korean expansion plans. Most items remain at the disclosure stage, and real capacity or employment impact still depends on formal approvals, construction, and equipment-install timelines.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
     </row>
   </sheetData>
@@ -687,7 +687,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="226" customHeight="1">
+    <row r="3" ht="210" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>01</t>
@@ -702,7 +702,7 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Malaysia AI-facility commitments and delivery milestones remain distinct
+            <t xml:space="preserve">Malaysia approves 27 data-center projects worth about US$55.4 billion
 </t>
           </r>
           <r>
@@ -711,20 +711,20 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>Bitdeer’s A201 in Malaysia still distinguishes site readiness in January 2027 from full deployment in April 2027, while Aolani’s disclosure is only a non-binding LOI covering up to 500 MW. Both cases show that AI-facility progress is measured separately by contracted coverage, site completion and power readiness, and cannot be treated as installed capacity. The critical milestones for an AI facility span GPUs, server racks, liquid cooling and site power. Company updates list an operating A101, a planned A201, group GPU utilization and future contracted revenue at the same time, which are distinct layers rather than one single operational figure. Bitdeer reports 95% September GPU utilization, but that does not equal A201’s actual monthly output; A201 still distinguishes readiness from full deployment. Aolani lists non-binding LOIs for up to 500 MW, which means the final customer uptake and power timeline are not yet defined. Public disclosure does not yet fully explain A201’s delivery conditions, which customers are already committed, or the gap between energization and revenue recognition. Those items remain contingent on formal delivery notices, power-availability statements and contractual terms. Location: Johor Bahru, Malaysia; A201 and A101 sites listed separately.</t>
+            <t>Regional coverage reviewed on October 21 says Malaysia has approved 27 additional data-center projects worth about US$55.4 billion. The figure reflects approvals and investment commitments rather than same-day energization, rack deployment, and commercial operations; supply-chain impact still depends on construction, substation, and tenant ramp timing. Data-center approvals affect server racks, power distribution, cooling, construction, and long-lead electrical equipment demand. For Taiwan and Southeast Asia, the first effect is an engineering and equipment-procurement window, followed later by actual tenant installation and operating revenue. “27 projects and US$55.4 billion” denotes approved pipeline scale, not directly live MW. Short-term impact still requires separating land progress, grid interconnection, MEP buildout, and contract maturity with tenants. Public reporting does not fully list energization dates, IT loads, or phased go-live points for each project, so approved totals cannot be converted directly into annual live capacity. Location: Malaysia (centered on the Peninsular data-center corridor, with Johor and Greater Kuala Lumpur as key areas).</t>
           </r>
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>For precision-power and measurement-equipment suppliers, the focus is not a single utilization number but whether the site can be delivered, energized and validated. If customer take-up and power milestones remain unresolved, equipment-purchase timing can be delayed, and those points must be checked alongside contract terms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="226" customHeight="1">
+          <t>For precision-power and measurement suppliers, this approval batch is a trackable engineering and energization pipeline rather than immediately recognizable equipment sales. The next checks are phased go-live timing, available grid headroom, and real tenant ramp speed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="210" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>02</t>
@@ -739,7 +739,7 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">MiTAC’s new-factory and expansion plan is public, but capacity timing is not yet defined
+            <t xml:space="preserve">Peninsular Malaysia data-center demand estimated at 8,391MW by 2030, with Johor above half
 </t>
           </r>
           <r>
@@ -748,16 +748,16 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>MiTAC disclosed approximately NT$12.62 billion in Taiwan investment covering a new Yangmei plant and expansions in Zhunan and Linkou, but did not publish the equipment-install timing or acceptance thresholds for each site. The project remains a planned capital expansion rather than an immediate shipped or live capacity figure. The package covers a new factory and expansion of existing lines, reflecting server, AI-related assembly and high-density power requirements. In supply-chain terms, this suggests expansion in racks, assembly and power-related demand, rather than a single mass-production site already fully online. The company did not disclose site-by-site build schedules, equipment lead times or power loads, so the disclosed investment cannot be equated directly with near-term shipments. Those details may appear in later filings, but current reading must keep plans and acceptance conditions separate. The investment, site and plant plans are public, but actual construction start dates, equipment installation dates and per-site capacity targets remain unpublished, so only the capital plan and expansion direction can be confirmed today. Location: Yangmei, Zhunan and Linkou, Taiwan; the disclosure refers to site plans.</t>
+            <t>October 21 reporting indicates Peninsular Malaysia data-center demand could reach 8,391MW by 2030, with Johor accounting for more than half. This is a demand estimate rather than current load; real supply-chain effects still depend on grid upgrades, interconnection approvals, and phased commissioning. Data-center demand usually appears first in requested capacity and interconnection planning, then later in usable IT load. If grid upgrades, substation expansion, and backup infrastructure progress are not synchronized, estimated demand will not immediately become deliverable capacity. This story focuses on regional demand and geographic concentration, not the prior day’s company-level contract coverage or single-site delivery milestones. The emphasis shifts from one-project operating metrics to system-level power pressure and infrastructure support. A complete public project-by-project list for energization and deployment timing is still unavailable, so 8,391MW should currently be treated as a scale indicator of demand. Location: Peninsular Malaysia (with Johor as the main concentration).</t>
           </r>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>For server and power-supply-chain firms, this type of investment mostly reflects medium-term line preparation rather than immediate shipment growth. The key is equipment lead times, facility energization and line acceptance; otherwise planned expansion can be mistaken for achieved capacity.</t>
+          <t>For precision-power and measurement suppliers, 8,391MW is potential design load, not immediately recognizable market volume. Order timing still depends on whether substation milestones, interconnection approvals, and tenant deployment phases align.</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">TPK and PTI packaging equipment and glass-substrate validation still center on pilot runs and customer acceptance
+            <t xml:space="preserve">Vietnam electronics expansion signals strengthen, with multi-billion-dollar intentions still pending execution
 </t>
           </r>
           <r>
@@ -785,16 +785,16 @@
               <color rgb="003B4A44"/>
               <sz val="11"/>
             </rPr>
-            <t>TPK outlines a two-year NT$6 billion TGV plan, while PTI discloses nearby equipment procurement and packaging-validation milestones. Both actions emphasize validation, scale-up and customer-fit, but they do not yet amount to production readiness, because equipment purchase, pilot production and customer acceptance are separate milestones. TGV, glass-substrate and analysis equipment sit on the critical path for advanced packaging and high-density power. These projects still revolve around pilot runs, equipment installation and line qualification, not mass-production contracts in place. Regional equipment purchases and factory planning certainly show continued investment, but outlay must be kept separate from actual production volume, yield improvement and customer acceptance. For the supply chain, technical capability still needs to be confirmed through actual samples and customer verification. Public information does not yet provide complete yield, equipment-utilization and conversion-rate data, so pilot-scale and planning figures cannot yet be treated as the start of commercial mass production. Location: Taiwan; involving packaging, glass-substrate and equipment-service test and engineering nodes.</t>
+            <t>Supply-chain coverage reviewed on October 21 highlights continued multi-billion-dollar investment intentions in Vietnam’s electronics and chip-testing chain, including Taiwanese and Korean expansion plans. Most items remain at the disclosure stage, and real capacity or employment impact still depends on formal approvals, construction, and equipment-install timelines. If Vietnam expansion plans are executed, they would affect testing, power systems, fixtures, automation, and adjacent materials demand. For Taiwan and Southeast Asia, the key is not one headline number but whether approvals and equipment deployment form a sustained cadence. This item shifts to cross-border investment signals in Vietnam’s electronics and testing chain, avoiding repetition of prior-day Malaysia facility and Taiwan single-company investment themes. The focus is on regional capacity migration and execution conditions. Public information still lacks full disclosure on final approvals, construction milestones, and production start points, so investment intentions cannot yet be treated as near-term available capacity. Location: Northern Vietnam electronics-manufacturing corridor, including test and packaging-related sites.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>For packaging and equipment suppliers, the significance of this type of investment lies in building technical and validation capability, not in having reached a mass-production threshold. The key question is whether yield, delivery and customer validation keep moving forward, not just the capital outlay total.</t>
+          <t>For precision-power and measurement suppliers, the value of Vietnam expansion signals is improved medium-term visibility, while timing remains tied to approvals and construction. The immediate priority is to track energization, test-line buildout, and customer onboarding order rather than translating intention values directly into short-term revenue assumptions.</t>
         </is>
       </c>
     </row>

</xml_diff>